<commit_message>
Add verified published supplements: Hugo 2016, Riaz 2017, Gide 2019
- data/supplements/{hugo2016,riaz2017,gide2019}/: raw publisher files (small
  committed; large .xls/.pdf/large .xlsx git-ignored, preserved locally with
  MD5 checksums) + cleaned per-sheet CSVs + per-cohort provenance READMEs.
- 26 tables extracted and validated against each paper:
  * Hugo: WES 140x, median 489 nsSNV, BRCA2 flag, IPRES gene sets, 25k-row MAF.
  * Riaz: 73 clinical, mut-load median 182 (paper 183), 28k-row MAF w/ Taf for
    clonality, longitudinal WES+RNA+TCR availability matrix, neoantigen catalog.
  * Gide: mono/combo clinical (105 patients; paper's 63/57 are biopsy-level),
    DE genes + KEGG-GSEA per arm. No WES (consistent w/ cBioPortal).
- Registry supplements sheet + workbook updated to reflect extracted/verified status.
</commit_message>
<xml_diff>
--- a/data/registry/DATASET_REGISTRY.xlsx
+++ b/data/registry/DATASET_REGISTRY.xlsx
@@ -19,40 +19,31 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">covariates!$A$1:$D$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">coverage_verified!$A$1:$O$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">rna_phenotypes!$A$1:$D$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">supplements!$A$1:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">supplements!$A$1:$H$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="220">
   <si>
     <t>Dataset Registry — evolutionary-rna-state</t>
   </si>
   <si>
-    <t>Melanoma immune-checkpoint-blockade cohorts assembled for reconstructing a latent evolutionary RNA-state.</t>
-  </si>
-  <si>
-    <t>Sheets:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  cohorts            — master table: 5 melanoma ICB cohorts, roles, RNA/WES availability, why included</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  rna_phenotypes     — the 6 thesis RNA phenotypes mapped to their data sources</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  covariates         — confounders-to-beat (TMB, purity, ploidy, clonality, composition) + benchmark signatures</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  supplements        — per-paper supplemental data inventory + access status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  coverage_verified  — per-cohort field coverage, pulled live from cBioPortal (real %, not estimates)</t>
-  </si>
-  <si>
-    <t>RNA raw reads (FASTQ): Gide + Riaz + Hugo (ENA). Variant calls (no raw exomes): Riaz/Hugo/Liu/DFCI via cBioPortal iAtlas.</t>
+    <t>Melanoma ICB cohorts for reconstructing a latent evolutionary RNA-state.</t>
+  </si>
+  <si>
+    <t>Sheets: cohorts | rna_phenotypes | covariates | supplements | coverage_verified</t>
+  </si>
+  <si>
+    <t>RNA raw reads (FASTQ): Gide + Riaz + Hugo (ENA).</t>
+  </si>
+  <si>
+    <t>Variant calls: Riaz/Hugo/Liu/DFCI (cBioPortal iAtlas).</t>
+  </si>
+  <si>
+    <t>Published supplements (verified &amp; extracted): Hugo, Riaz, Gide -&gt; data/supplements/.</t>
   </si>
   <si>
     <t>Generated in-session during the hackathon. Public data only.</t>
@@ -451,109 +442,190 @@
     <t>role_in_analysis</t>
   </si>
   <si>
-    <t>Riaz 2017</t>
-  </si>
-  <si>
-    <t>Hugo 2016</t>
-  </si>
-  <si>
-    <t>Gide 2019</t>
-  </si>
-  <si>
-    <t>DFCI 2019</t>
-  </si>
-  <si>
-    <t>all iAtlas</t>
+    <t>Cell, PMID 26997480</t>
+  </si>
+  <si>
+    <t>Cell, PMID 29033130</t>
+  </si>
+  <si>
+    <t>Cancer Cell, PMID 30753825</t>
+  </si>
+  <si>
+    <t>S1A</t>
+  </si>
+  <si>
+    <t>S1B</t>
+  </si>
+  <si>
+    <t>S1C</t>
+  </si>
+  <si>
+    <t>S1D</t>
+  </si>
+  <si>
+    <t>S1E</t>
+  </si>
+  <si>
+    <t>S2A</t>
+  </si>
+  <si>
+    <t>S2B</t>
+  </si>
+  <si>
+    <t>S2C</t>
   </si>
   <si>
     <t>Table S1</t>
   </si>
   <si>
-    <t>Table S2/S3</t>
-  </si>
-  <si>
-    <t>PyClone output</t>
-  </si>
-  <si>
-    <t>Table S1A/B/C</t>
-  </si>
-  <si>
-    <t>Table S2B</t>
-  </si>
-  <si>
-    <t>mass cytometry</t>
-  </si>
-  <si>
-    <t>cBioPortal</t>
-  </si>
-  <si>
-    <t>cBioPortal API</t>
-  </si>
-  <si>
-    <t>WES sample metadata &amp; depth (150x)</t>
-  </si>
-  <si>
-    <t>per-patient mutation &amp; neoantigen load</t>
-  </si>
-  <si>
-    <t>per-SNV CCF, clonal vs subclonal</t>
-  </si>
-  <si>
-    <t>WES 140x, 489 nsSNV, neoepitope loads</t>
-  </si>
-  <si>
-    <t>IPRES signature gene sets (GSVA)</t>
-  </si>
-  <si>
-    <t>EOMES+CD69+CD45RO+ effector-memory T-cell sig</t>
-  </si>
-  <si>
-    <t>clonal/subclonal counts, purity, ploidy, CNA</t>
-  </si>
-  <si>
-    <t>per-category neoantigen, TMB, response, survival, TIDE</t>
-  </si>
-  <si>
-    <t>Cell mmc (publisher)</t>
-  </si>
-  <si>
-    <t>Cancer Cell mmc</t>
-  </si>
-  <si>
-    <t>cBioPortal API (pulled)</t>
-  </si>
-  <si>
-    <t>needed only for raw-CCF; else iAtlas covers</t>
-  </si>
-  <si>
-    <t>iAtlas MAF covers most</t>
-  </si>
-  <si>
-    <t>request if phylogeny figure needed</t>
-  </si>
-  <si>
-    <t>iAtlas MAF covers</t>
-  </si>
-  <si>
-    <t>reconstruct signature for benchmark</t>
-  </si>
-  <si>
-    <t>optional composition benchmark</t>
-  </si>
-  <si>
-    <t>IN HAND</t>
+    <t>Table S2</t>
+  </si>
+  <si>
+    <t>Table S3</t>
+  </si>
+  <si>
+    <t>Table S4</t>
+  </si>
+  <si>
+    <t>Table S5A</t>
+  </si>
+  <si>
+    <t>Table S5B</t>
+  </si>
+  <si>
+    <t>Table S6A</t>
+  </si>
+  <si>
+    <t>Table S6B</t>
+  </si>
+  <si>
+    <t>Table S6C</t>
+  </si>
+  <si>
+    <t>Table S6D</t>
+  </si>
+  <si>
+    <t>Table S1. PD-1 Patient</t>
+  </si>
+  <si>
+    <t>Table S2. PD-1+CTLA-4 patients</t>
+  </si>
+  <si>
+    <t>Table S3. PD1-DEgenes</t>
+  </si>
+  <si>
+    <t>Table S4. PD1_GSEA-KEGG</t>
+  </si>
+  <si>
+    <t>Table S5. PD1+CTLA4-DEgenes</t>
+  </si>
+  <si>
+    <t>Table S6. ipiPD1_GSEA-KEGG</t>
+  </si>
+  <si>
+    <t>Table S7. Venn_PRE</t>
+  </si>
+  <si>
+    <t>Table S8. Venn_EDT</t>
+  </si>
+  <si>
+    <t>clean/hugo2016_S1A.csv</t>
+  </si>
+  <si>
+    <t>clean/hugo2016_S1B.csv</t>
+  </si>
+  <si>
+    <t>clean/hugo2016_S1C.csv</t>
+  </si>
+  <si>
+    <t>clean/hugo2016_S1D.csv</t>
+  </si>
+  <si>
+    <t>clean/hugo2016_S1E.csv</t>
+  </si>
+  <si>
+    <t>clean/hugo2016_S2A.csv</t>
+  </si>
+  <si>
+    <t>clean/hugo2016_S2B.csv</t>
+  </si>
+  <si>
+    <t>clean/hugo2016_S2C.csv</t>
+  </si>
+  <si>
+    <t>clean/riaz2017_S1.csv</t>
+  </si>
+  <si>
+    <t>clean/riaz2017_S2.csv</t>
+  </si>
+  <si>
+    <t>clean/riaz2017_S3.csv</t>
+  </si>
+  <si>
+    <t>clean/riaz2017_S4.csv</t>
+  </si>
+  <si>
+    <t>clean/riaz2017_S5A.csv</t>
+  </si>
+  <si>
+    <t>clean/riaz2017_S5B.csv</t>
+  </si>
+  <si>
+    <t>clean/riaz2017_S6A.csv</t>
+  </si>
+  <si>
+    <t>clean/riaz2017_S6B.csv</t>
+  </si>
+  <si>
+    <t>clean/riaz2017_S6C.csv</t>
+  </si>
+  <si>
+    <t>clean/riaz2017_S6D.csv</t>
+  </si>
+  <si>
+    <t>clean/gide2019_S1_PD1_clinical.csv</t>
+  </si>
+  <si>
+    <t>clean/gide2019_S2_comboclinical.csv</t>
+  </si>
+  <si>
+    <t>clean/gide2019_S3_PD1_DEgenes.csv</t>
+  </si>
+  <si>
+    <t>clean/gide2019_S4_PD1_KEGG.csv</t>
+  </si>
+  <si>
+    <t>clean/gide2019_S5_combo_DEgenes.csv</t>
+  </si>
+  <si>
+    <t>clean/gide2019_S6_combo_KEGG.csv</t>
+  </si>
+  <si>
+    <t>clean/gide2019_S7_Venn_PRE.csv</t>
+  </si>
+  <si>
+    <t>clean/gide2019_S8_Venn_EDT.csv</t>
+  </si>
+  <si>
+    <t>IN HAND — extracted &amp; verified</t>
   </si>
   <si>
     <t>cohort</t>
   </si>
   <si>
-    <t>item</t>
-  </si>
-  <si>
-    <t>contents</t>
-  </si>
-  <si>
-    <t>access</t>
+    <t>citation</t>
+  </si>
+  <si>
+    <t>sheet</t>
+  </si>
+  <si>
+    <t>clean_csv</t>
+  </si>
+  <si>
+    <t>rows</t>
+  </si>
+  <si>
+    <t>cols</t>
   </si>
   <si>
     <t>99%</t>
@@ -997,10 +1069,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="110.7109375" customWidth="1"/>
+    <col min="1" max="1" width="105.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
@@ -1017,46 +1089,31 @@
       <c r="A3" s="2"/>
     </row>
     <row r="4" spans="1:1">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:1">
-      <c r="A5" s="2" t="s">
-        <v>3</v>
-      </c>
+      <c r="A5" s="2"/>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1">
-      <c r="A10" s="2"/>
-    </row>
-    <row r="11" spans="1:1">
-      <c r="A11" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1">
-      <c r="A12" s="2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1090,84 +1147,84 @@
   <sheetData>
     <row r="1" spans="1:19">
       <c r="A1" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="R1" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="S1" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="R1" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:19">
       <c r="A2" s="3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D2" s="3">
         <v>30753825</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H2" s="3">
         <v>91</v>
@@ -1179,54 +1236,54 @@
         <v>18</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="L2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="M2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="M2" s="3" t="s">
-        <v>41</v>
-      </c>
       <c r="N2" s="3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D3" s="3">
         <v>29033130</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H3" s="3">
         <v>109</v>
@@ -1238,54 +1295,54 @@
         <v>58</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D4" s="3">
         <v>26997480</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>26</v>
-      </c>
       <c r="G4" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H4" s="3">
         <v>24</v>
@@ -1297,54 +1354,54 @@
         <v>0</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="M4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N4" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="N4" s="3" t="s">
-        <v>44</v>
-      </c>
       <c r="O4" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:19">
       <c r="A5" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5" s="3">
         <v>31792460</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H5" s="3">
         <v>0</v>
@@ -1356,54 +1413,54 @@
         <v>0</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="S5" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:19">
       <c r="A6" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="D6" s="3">
         <v>31792460</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H6" s="3">
         <v>0</v>
@@ -1415,31 +1472,31 @@
         <v>0</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="R6" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1461,100 +1518,100 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>107</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>102</v>
-      </c>
       <c r="D5" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1576,114 +1633,114 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>137</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -1694,171 +1751,723 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="55.7109375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="25.7109375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="45.7109375" style="3" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="32.7109375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="37.7109375" style="3" customWidth="1"/>
+    <col min="6" max="6" width="7.7109375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" style="3" customWidth="1"/>
+    <col min="8" max="8" width="32.7109375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:8">
       <c r="A1" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F2" s="3">
+        <v>42</v>
+      </c>
+      <c r="G2" s="3">
+        <v>22</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F3" s="3">
+        <v>39</v>
+      </c>
+      <c r="G3" s="3">
+        <v>45</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="F4" s="3">
+        <v>37</v>
+      </c>
+      <c r="G4" s="3">
+        <v>6</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="F5" s="3">
+        <v>25393</v>
+      </c>
+      <c r="G5" s="3">
+        <v>17</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="F6" s="3">
+        <v>36</v>
+      </c>
+      <c r="G6" s="3">
+        <v>11</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="F7" s="3">
+        <v>693</v>
+      </c>
+      <c r="G7" s="3">
+        <v>7</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="F8" s="3">
+        <v>72</v>
+      </c>
+      <c r="G8" s="3">
+        <v>7</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="F9" s="3">
+        <v>19</v>
+      </c>
+      <c r="G9" s="3">
+        <v>3</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="C2" s="3" t="s">
+      <c r="F10" s="3">
+        <v>68</v>
+      </c>
+      <c r="G10" s="3">
+        <v>40</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="F11" s="3">
+        <v>73</v>
+      </c>
+      <c r="G11" s="3">
+        <v>12</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="F12" s="3">
+        <v>28589</v>
+      </c>
+      <c r="G12" s="3">
+        <v>11</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="F13" s="3">
+        <v>80</v>
+      </c>
+      <c r="G13" s="3">
+        <v>7</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="F14" s="3">
+        <v>41477</v>
+      </c>
+      <c r="G14" s="3">
+        <v>8</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E15" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F15" s="3">
+        <v>4492</v>
+      </c>
+      <c r="G15" s="3">
+        <v>8</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="F16" s="3">
+        <v>189</v>
+      </c>
+      <c r="G16" s="3">
+        <v>6</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="F17" s="3">
+        <v>1384</v>
+      </c>
+      <c r="G17" s="3">
+        <v>6</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="F18" s="3">
+        <v>475</v>
+      </c>
+      <c r="G18" s="3">
+        <v>6</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="F19" s="3">
+        <v>2670</v>
+      </c>
+      <c r="G19" s="3">
+        <v>6</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="F20" s="3">
+        <v>54</v>
+      </c>
+      <c r="G20" s="3">
+        <v>15</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="F21" s="3">
+        <v>51</v>
+      </c>
+      <c r="G21" s="3">
+        <v>15</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="F22" s="3">
+        <v>310</v>
+      </c>
+      <c r="G22" s="3">
+        <v>14</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E23" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="F23" s="3">
+        <v>12</v>
+      </c>
+      <c r="G23" s="3">
+        <v>7</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F24" s="3">
+        <v>328</v>
+      </c>
+      <c r="G24" s="3">
+        <v>13</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="F25" s="3">
+        <v>11</v>
+      </c>
+      <c r="G25" s="3">
+        <v>7</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="E3" s="3" t="s">
+      <c r="E26" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="F26" s="3">
+        <v>123</v>
+      </c>
+      <c r="G26" s="3">
+        <v>3</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>171</v>
+      <c r="E27" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F27" s="3">
+        <v>133</v>
+      </c>
+      <c r="G27" s="3">
+        <v>3</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E9"/>
+  <autoFilter ref="A1:H27"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1886,284 +2495,284 @@
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="4" t="s">
-        <v>172</v>
+        <v>194</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>182</v>
+        <v>206</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>183</v>
+        <v>207</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>184</v>
+        <v>208</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>186</v>
+        <v>210</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>187</v>
+        <v>211</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>188</v>
+        <v>212</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>189</v>
+        <v>213</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>190</v>
+        <v>214</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>191</v>
+        <v>215</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>192</v>
+        <v>216</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>193</v>
+        <v>217</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>194</v>
+        <v>218</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>195</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2" spans="1:15">
       <c r="A2" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B2" s="3">
         <v>144</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:15">
       <c r="A3" s="3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B3" s="3">
         <v>91</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B4" s="3">
         <v>27</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>180</v>
+        <v>204</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B5" s="3">
         <v>122</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B6" s="3">
         <v>107</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>181</v>
+        <v>205</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>